<commit_message>
Update multiple Python scripts and README; added error handling, improved functionality, and removed unused files.
</commit_message>
<xml_diff>
--- a/17.날씨 예보 프로그램/날씨저장.xlsx
+++ b/17.날씨 예보 프로그램/날씨저장.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -446,24 +446,24 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2023-03-06</t>
+          <t>2025-09-27</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>20:06:51</t>
+          <t>16:40:09</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>scattered clouds</t>
+          <t>overcast clouds</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>8.66</v>
+        <v>26.35</v>
       </c>
       <c r="E2" t="n">
-        <v>7.87</v>
+        <v>26.35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>